<commit_message>
changes position after add a new data at excel file
</commit_message>
<xml_diff>
--- a/Source data.xlsx
+++ b/Source data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Shimul Mama's Project V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461D9975-8B92-42AF-A5F7-555605327B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F89467-1182-4700-B15F-8446497F7913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E9D45CA4-9EFC-465D-85A4-FCF3CFEE9A51}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data!$B$1:$M$441</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3092" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3092" uniqueCount="229">
   <si>
     <t>OrderNo</t>
   </si>
@@ -716,6 +715,9 @@
   </si>
   <si>
     <t>Unit</t>
+  </si>
+  <si>
+    <t>abc</t>
   </si>
 </sst>
 </file>
@@ -8120,7 +8122,7 @@
         <v>270040</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>115</v>
+        <v>228</v>
       </c>
       <c r="D185" s="4" t="s">
         <v>85</v>

</xml_diff>